<commit_message>
fix: deleted unneeded column
</commit_message>
<xml_diff>
--- a/+AGMA/form_factor_table.xlsx
+++ b/+AGMA/form_factor_table.xlsx
@@ -14,21 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>NumberOfTeeth_N_</t>
   </si>
   <si>
     <t>LewisFormFactor_Y_</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>← 피니언 (N=16)</t>
-  </si>
-  <si>
-    <t>← N=48 보간 기준점</t>
   </si>
   <si>
     <t>Source: Shigley's Mechanical Engineering Design, Table 14-2</t>
@@ -39,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -55,8 +46,14 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -123,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -131,55 +128,37 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
   </cellXfs>
@@ -484,12 +463,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="17" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="18" width="24.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="19" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="24.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -499,252 +477,216 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="3">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0.245</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="3">
+        <v>13</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.261</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="3">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.277</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="3">
+        <v>15</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="5">
+        <v>16</v>
+      </c>
+      <c r="B6" s="6">
+        <v>0.296</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="3">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0.303</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="3">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4">
+        <v>0.309</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="3">
+        <v>19</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.314</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="3">
+        <v>20</v>
+      </c>
+      <c r="B10" s="4">
+        <v>0.322</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="3">
+        <v>21</v>
+      </c>
+      <c r="B11" s="4">
+        <v>0.328</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="3">
+        <v>22</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0.331</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="3">
+        <v>24</v>
+      </c>
+      <c r="B13" s="4">
+        <v>0.337</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="3">
+        <v>26</v>
+      </c>
+      <c r="B14" s="4">
+        <v>0.346</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="3">
+        <v>28</v>
+      </c>
+      <c r="B15" s="4">
+        <v>0.353</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="3">
+        <v>30</v>
+      </c>
+      <c r="B16" s="4">
+        <v>0.359</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="3">
+        <v>34</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0.371</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="3">
+        <v>38</v>
+      </c>
+      <c r="B18" s="4">
+        <v>0.384</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="20.25">
+      <c r="A19" s="7">
+        <v>43</v>
+      </c>
+      <c r="B19" s="8">
+        <v>0.397</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="20.25">
+      <c r="A20" s="7">
+        <v>50</v>
+      </c>
+      <c r="B20" s="8">
+        <v>0.409</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="3">
+        <v>60</v>
+      </c>
+      <c r="B21" s="4">
+        <v>0.422</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="3">
+        <v>75</v>
+      </c>
+      <c r="B22" s="4">
+        <v>0.435</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="3">
+        <v>100</v>
+      </c>
+      <c r="B23" s="4">
+        <v>0.447</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="3">
+        <v>150</v>
+      </c>
+      <c r="B24" s="4">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="3">
+        <v>300</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.472</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="3">
+        <v>400</v>
+      </c>
+      <c r="B26" s="4">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="9"/>
+      <c r="B27" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="11" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="4">
-        <v>12</v>
-      </c>
-      <c r="B2" s="5">
-        <v>0.245</v>
-      </c>
-      <c r="C2" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="4">
-        <v>13</v>
-      </c>
-      <c r="B3" s="5">
-        <v>0.261</v>
-      </c>
-      <c r="C3" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="4">
-        <v>14</v>
-      </c>
-      <c r="B4" s="5">
-        <v>0.277</v>
-      </c>
-      <c r="C4" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="4">
-        <v>15</v>
-      </c>
-      <c r="B5" s="5">
-        <v>0.29</v>
-      </c>
-      <c r="C5" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
-      <c r="A6" s="7">
-        <v>16</v>
-      </c>
-      <c r="B6" s="8">
-        <v>0.296</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="4">
-        <v>17</v>
-      </c>
-      <c r="B7" s="5">
-        <v>0.303</v>
-      </c>
-      <c r="C7" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="4">
-        <v>18</v>
-      </c>
-      <c r="B8" s="5">
-        <v>0.309</v>
-      </c>
-      <c r="C8" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="4">
-        <v>19</v>
-      </c>
-      <c r="B9" s="5">
-        <v>0.314</v>
-      </c>
-      <c r="C9" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="4">
-        <v>20</v>
-      </c>
-      <c r="B10" s="5">
-        <v>0.322</v>
-      </c>
-      <c r="C10" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="4">
-        <v>21</v>
-      </c>
-      <c r="B11" s="5">
-        <v>0.328</v>
-      </c>
-      <c r="C11" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="4">
-        <v>22</v>
-      </c>
-      <c r="B12" s="5">
-        <v>0.331</v>
-      </c>
-      <c r="C12" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="4">
-        <v>24</v>
-      </c>
-      <c r="B13" s="5">
-        <v>0.337</v>
-      </c>
-      <c r="C13" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="4">
-        <v>26</v>
-      </c>
-      <c r="B14" s="5">
-        <v>0.346</v>
-      </c>
-      <c r="C14" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="4">
-        <v>28</v>
-      </c>
-      <c r="B15" s="5">
-        <v>0.353</v>
-      </c>
-      <c r="C15" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="4">
-        <v>30</v>
-      </c>
-      <c r="B16" s="5">
-        <v>0.359</v>
-      </c>
-      <c r="C16" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="4">
-        <v>34</v>
-      </c>
-      <c r="B17" s="5">
-        <v>0.371</v>
-      </c>
-      <c r="C17" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="4">
-        <v>38</v>
-      </c>
-      <c r="B18" s="5">
-        <v>0.384</v>
-      </c>
-      <c r="C18" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="20.25">
-      <c r="A19" s="10">
-        <v>43</v>
-      </c>
-      <c r="B19" s="11">
-        <v>0.397</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="20.25">
-      <c r="A20" s="10">
-        <v>50</v>
-      </c>
-      <c r="B20" s="11">
-        <v>0.409</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="4">
-        <v>60</v>
-      </c>
-      <c r="B21" s="5">
-        <v>0.422</v>
-      </c>
-      <c r="C21" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="4">
-        <v>75</v>
-      </c>
-      <c r="B22" s="5">
-        <v>0.435</v>
-      </c>
-      <c r="C22" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="4">
-        <v>100</v>
-      </c>
-      <c r="B23" s="5">
-        <v>0.447</v>
-      </c>
-      <c r="C23" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="4">
-        <v>150</v>
-      </c>
-      <c r="B24" s="5">
-        <v>0.46</v>
-      </c>
-      <c r="C24" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="4">
-        <v>300</v>
-      </c>
-      <c r="B25" s="5">
-        <v>0.472</v>
-      </c>
-      <c r="C25" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="4">
-        <v>400</v>
-      </c>
-      <c r="B26" s="5">
-        <v>0.48</v>
-      </c>
-      <c r="C26" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="15"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="15"/>
+      <c r="B28" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>